<commit_message>
chore: update dataset template for posyandu data entry
</commit_message>
<xml_diff>
--- a/WD/frontend/public/template_pengisian_dataset_posyandu.xlsx
+++ b/WD/frontend/public/template_pengisian_dataset_posyandu.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="23">
   <si>
     <t>No</t>
   </si>
@@ -75,6 +75,33 @@
   </si>
   <si>
     <t>NORMAL(0) STUNTING (1)</t>
+  </si>
+  <si>
+    <t>TB(kg)</t>
+  </si>
+  <si>
+    <t>BB(cm)</t>
+  </si>
+  <si>
+    <t>Juni</t>
+  </si>
+  <si>
+    <t>Juli</t>
+  </si>
+  <si>
+    <t>Agustus</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>November</t>
+  </si>
+  <si>
+    <t>Desember</t>
   </si>
 </sst>
 </file>
@@ -151,13 +178,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -485,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q92"/>
+  <dimension ref="A1:AE92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
@@ -493,59 +523,87 @@
     <col min="3" max="3" width="14.28515625" customWidth="1"/>
     <col min="4" max="4" width="14.85546875" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" customWidth="1"/>
-    <col min="17" max="17" width="24.140625" customWidth="1"/>
+    <col min="31" max="31" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="4"/>
-      <c r="I1" s="3" t="s">
+      <c r="H1" s="5"/>
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4"/>
-      <c r="K1" s="3" t="s">
+      <c r="J1" s="5"/>
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="3" t="s">
+      <c r="L1" s="5"/>
+      <c r="M1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="3" t="s">
+      <c r="N1" s="5"/>
+      <c r="O1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="5" t="s">
+      <c r="P1" s="5"/>
+      <c r="Q1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="5"/>
+      <c r="S1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" s="5"/>
+      <c r="U1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="V1" s="5"/>
+      <c r="W1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z1" s="5"/>
+      <c r="AA1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB1" s="5"/>
+      <c r="AC1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD1" s="5"/>
+      <c r="AE1" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="5"/>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="6"/>
       <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
@@ -576,74 +634,116 @@
       <c r="P2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="Q2" s="5"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE2" s="6"/>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -1029,9 +1129,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="19">
+    <mergeCell ref="AC1:AD1"/>
+    <mergeCell ref="AA1:AB1"/>
+    <mergeCell ref="Y1:Z1"/>
     <mergeCell ref="O1:P1"/>
-    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="AE1:AE2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
@@ -1042,6 +1145,10 @@
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="M1:N1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="W1:X1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>